<commit_message>
Amber: RheinWeg: add Oberursel_steuerberater.xlsx and Oberursel_dachdecker.xlsx
</commit_message>
<xml_diff>
--- a/P(Path)/RP(Rhine-Path)/Oberursel_dachdecker.xlsx
+++ b/P(Path)/RP(Rhine-Path)/Oberursel_dachdecker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yanghan/CODE/GitHub/Amber2/P(Path)/RP(Rhine-Path)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FFBE1F55-2822-5146-9919-5CAA8A4E1AF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76C0B1B3-6BDE-C248-AE88-6485E0DA2D94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4400" yWindow="3140" windowWidth="60160" windowHeight="31440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16680" yWindow="1980" windowWidth="39220" windowHeight="27800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oberursel (Taunus)" sheetId="1" r:id="rId1"/>
@@ -1511,7 +1511,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="53" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
@@ -3713,5 +3713,6 @@
     <mergeCell ref="A1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>